<commit_message>
ADMIN: cambia archivo excel plantilla dni
</commit_message>
<xml_diff>
--- a/public/assets/backend/docs/plantilla_import_dni.xlsx
+++ b/public/assets/backend/docs/plantilla_import_dni.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>DNI</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>ID_REGION</t>
+  </si>
+  <si>
+    <t>APELLIDO</t>
   </si>
 </sst>
 </file>
@@ -479,7 +482,7 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -493,7 +496,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>

</xml_diff>